<commit_message>
Phase 2J hoàn tất.
- Final Business Sign-off:
  - total_signoff_items = 3
  - approved_count = 3
  - proposed_status = FINAL_BUSINESS_SIGNOFF_APPROVED
- Ba item được duyệt chỉ cho bước thiết kế executor:
  - CHINT NXM-63S
  - CHINT NXM-125S
  - CHINT NXM-250S
- ready_for_execution = FALSE
- ready_for_write_to_main_pipeline = FALSE
</commit_message>
<xml_diff>
--- a/feasibility_outputs/profile_commit_gate/profile_commit_gate_review.xlsx
+++ b/feasibility_outputs/profile_commit_gate/profile_commit_gate_review.xlsx
@@ -54,8 +54,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2F0D9"/>
+        <bgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -460,7 +460,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,7 +483,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>PENDING_HUMAN_APPROVAL</t>
+          <t>APPROVED_FOR_NEXT_PHASE_DESIGN_ONLY</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Human candidate review</t>
+          <t>Phase 2E write simulation design</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -565,7 +565,11 @@
           <t>approved_by</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Project Owner</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -626,7 +630,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6b28f78bb1ca9325f4ab2c94cfd0e519d88b01a5972ee815e8515b6fa21c583b</t>
+          <t>23cdc35feb076554f5cd5280759fa3dbbdfac5d0d23449f26feb08f41602c648</t>
         </is>
       </c>
     </row>
@@ -650,7 +654,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>295942a0418064766fb63bc7c267d609b3603ea57919141e3f574a8379b74e8a</t>
+          <t>217f62e5d3e1a4af5b1e30ae875de7740ace76805ef9d8c0774650ed57629b69</t>
         </is>
       </c>
     </row>

</xml_diff>